<commit_message>
Bump more projects into medium difficulty by narrowing easy's range
Raw difficulty values skew lower after the cospecies-discount rework
(simulated: ~63% of generated projects landed "easy"). Moving the
easy/medium boundary value (5) from easy into medium shifted that to
~45% easy / ~50% medium, with hard's share untouched - tier_for_difficulty
is the single source RANGES feeds, so this cascades into the displayed
badge, OR/multiplier frequency during generation, and acceptance checks
consistently.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Predefined projects.xlsx
+++ b/data/Predefined projects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Zoo_tycoon_generatorv2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236B3A94-4835-40DE-909C-76313D930D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E9C03D-90CA-40C0-B2D1-EE445EBE1612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -435,7 +435,7 @@
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" customWidth="1"/>
     <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="24.5703125" customWidth="1"/>
+    <col min="4" max="4" width="32.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>